<commit_message>
case study slides refining
</commit_message>
<xml_diff>
--- a/Case_Studies_Master_IDed.xlsx
+++ b/Case_Studies_Master_IDed.xlsx
@@ -391,7 +391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I161"/>
+  <dimension ref="A1:I176"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="4" min="1" max="1"/>
@@ -8131,6 +8131,711 @@
       </c>
       <c r="I161" s="7" t="n"/>
     </row>
+    <row r="162">
+      <c r="A162" s="4" t="inlineStr">
+        <is>
+          <t>MSS081</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C162" s="4" t="inlineStr">
+        <is>
+          <t>Technology &amp; IT Services, Sales and Commercial Operations, ai-powered, pricing, estimation, engine, requirement, configuration, effort, timeline, dynamic, margin</t>
+        </is>
+      </c>
+      <c r="D162" s="4" t="inlineStr">
+        <is>
+          <t>AI-POWERED PRICING AND ESTIMATION ENGINE</t>
+        </is>
+      </c>
+      <c r="E162" s="4" t="inlineStr">
+        <is>
+          <t>As the service portfolio expanded, project estimation at this IT services firm had become a function of who was in the room - experienced individuals applying personal judgment to spreadsheets, disconnected cost models, and partial delivery histories. Quotes for similar engagements carried wildly inconsistent margins, and the gap between estimated and actual effort only became visible months into delivery. Historical project knowledge existed but sat in closed files and individual memories, inaccessible at the moment a new quote needed to be built. By the time a proposal reached a client, its commercial accuracy was already a risk the business had silently accepted.</t>
+        </is>
+      </c>
+      <c r="F162" s="4" t="inlineStr">
+        <is>
+          <t>An AI-powered pricing and estimation engine was deployed to systematically replace judgment-based quoting with a platform that learns from every completed engagement. It ingests historical delivery data, project characteristics, and resource patterns, producing effort estimates, timelines, staffing requirements, and risk-adjusted pricing in under five minutes from requirement inputs. Configurable business rules enforce margin thresholds, discount governance, and risk adjustments automatically, so every quote reflects the same commercial logic regardless of who built it. Teams now work from an evidence-based starting point and can run real-time what-if scenarios across scope and delivery model before committing to a price.</t>
+        </is>
+      </c>
+      <c r="G162" s="4" t="inlineStr">
+        <is>
+          <t>Requirement Configuration Engine: Guided questionnaires capture scope, complexity, and constraints, automatically configuring project parameters without manual interpretation.
+AI Effort and Timeline Estimation: Analyzes historical delivery patterns to predict effort, staffing, and timelines with accuracy that improves as the model trains on outcomes.
+Dynamic Pricing and Margin Control: Applies pricing rules, margin thresholds, and risk adjustments automatically, enforcing commercial governance across every quote.
+Scenario Planning and Profitability Comparison: Real-time what-if analysis across scope, delivery model, and resource mix with instant cost and margin comparison.
+Estimation Governance and Standardization: Enforces consistent pricing logic across all sales and delivery teams, eliminating variance driven by individual judgment.
+Continuous Model Retraining: Actual delivery outcomes retrain the estimation models with every completed project, compounding accuracy over time.</t>
+        </is>
+      </c>
+      <c r="H162" s="4" t="inlineStr">
+        <is>
+          <t>90%+ reduction in manual estimation effort per quote; Under 5 minutes from requirements input to complete, commercially governed project quote; Pricing decisions shifted from individual judgment to evidence-based governance, reducing margin leakage across the portfolio</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="4" t="inlineStr">
+        <is>
+          <t>MSS082</t>
+        </is>
+      </c>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C163" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Energy and Utilities Management, plant, energy, utilities, intelligence, asset-level, dashboards, utility, anomaly, detection, off-shift</t>
+        </is>
+      </c>
+      <c r="D163" s="4" t="inlineStr">
+        <is>
+          <t>PLANT ENERGY AND UTILITIES INTELLIGENCE</t>
+        </is>
+      </c>
+      <c r="E163" s="4" t="inlineStr">
+        <is>
+          <t>At this manufacturer, energy was the second-largest controllable cost on site - and it was being managed monthly, in arrears, from utility bills. There was no visibility into where energy was actually being consumed or wasted at the asset level across motors, chillers, compressors, HVAC, and process utilities. A drifting chiller, a stuck valve, or a conveyor left running off-shift could go unnoticed for weeks before the next bill made the loss visible. Teams had no way to compare consumption across lines, shifts, or sites, and sustainability targets were tracked on spreadsheets that nobody fully trusted.</t>
+        </is>
+      </c>
+      <c r="F163" s="4" t="inlineStr">
+        <is>
+          <t>A non-intrusive energy intelligence layer was deployed directly over the plant's existing meters, sub-meters, and SCADA historian tags, requiring no new process equipment and no writes to any control system. It delivered real-time consumption dashboards at asset, line, shift, and site level, with ML anomaly detection running continuously on motor, chiller, compressor, and HVAC signatures. Prescriptive load-balancing and peak-shaving recommendations were tied to the production schedule, and engineering alerts were routed automatically when corrective action was needed. The model was templatized after the lead-site pilot for rapid rollout across the remaining 8 plants.</t>
+        </is>
+      </c>
+      <c r="G163" s="4" t="inlineStr">
+        <is>
+          <t>Asset-Level Energy Dashboards: Real-time consumption visibility by asset, line, shift, and site, replacing monthly bill-based tracking with continuous intelligence.
+Utility Anomaly Detection: ML monitors motor, chiller, compressor, and HVAC signatures continuously, flagging drift within hours rather than weeks.
+Off-Shift Waste Detection: Pattern recognition identifies recurring inefficiencies and equipment running outside production windows across every shift.
+Peak Demand Management: Prescriptive load-balancing and peak-shaving recommendations tied directly to the production schedule.
+Engineering Alert Routing: Automated alerts sent to the responsible engineer the moment an anomaly crosses threshold, enabling same-day corrective action.
+Network Rollout Template: Standardized deployment model enabling rapid replication across all remaining sites after lead-site pilot validation.</t>
+        </is>
+      </c>
+      <c r="H163" s="4" t="inlineStr">
+        <is>
+          <t>11-13% reduction in energy cost on addressed scope in year 1; Anomaly detection-to-action cycle cut from weeks to under 24 hours; 100% asset-level energy visibility achieved, from a plant-level-only baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="4" t="inlineStr">
+        <is>
+          <t>MSS083</t>
+        </is>
+      </c>
+      <c r="B164" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C164" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Operational Excellence, ai-led, savings, opportunity, discovery, cross-system, data, ingestion, common, asset, model</t>
+        </is>
+      </c>
+      <c r="D164" s="4" t="inlineStr">
+        <is>
+          <t>AI-LED SAVINGS OPPORTUNITY DISCOVERY</t>
+        </is>
+      </c>
+      <c r="E164" s="4" t="inlineStr">
+        <is>
+          <t>Savings projects at this company were surfaced through periodic energy audits and kaizen events - slow, episodic, and entirely dependent on a small group of experts who could only be in one place at a time. Operational data sat in silos that never spoke to each other: energy meters, SCADA historian, MES, maintenance systems, and ERP each held a piece of the picture, but no one could see across all of them at once. Losses went invisible until they surfaced in month-end variance, and by then the decisions that caused them were weeks old. Leadership had no ranked, ROI-prioritized view of where to act - only the projects whoever happened to audit last thought were worth pursuing.</t>
+        </is>
+      </c>
+      <c r="F164" s="4" t="inlineStr">
+        <is>
+          <t>A read-only discovery layer was deployed connecting all existing plant systems without touching controls or replacing any platform. It normalized raw operational data to a common asset, line, and product model with per-tonne denominators, enabling shift-to-shift, line-to-line, and site-to-site benchmarking that had never existed before. ML loss detection surfaced deviation hotspots - assets running hot, leaks, changeover overruns, scrap clusters - and quantified each one in energy units, waste weight, downtime hours, and currency simultaneously. Plant engineers reviewed and validated the backlog before any project was committed, keeping human judgment in the prioritization decision.</t>
+        </is>
+      </c>
+      <c r="G164" s="4" t="inlineStr">
+        <is>
+          <t>Cross-System Data Ingestion: Read-only connection across energy, SCADA historian, MES, CMMS, and ERP with no control system changes required.
+Common Asset Model Normalization: Data normalized to asset, line, and product level with per-tonne denominators enabling true like-for-like comparison.
+ML Loss Detection: Identifies deviation hotspots across assets running hot, leaks, changeover overruns, and scrap clusters continuously.
+Multi-Dimensional Loss Quantification: Every identified loss expressed in energy units, waste weight, downtime hours, and currency in a single view.
+ROI-Ranked Savings Backlog: Projects ranked by financial return and implementation effort, validated with plant engineers before entering the action queue.
+Continuous Pipeline Refresh: Backlog updated continuously from live operational data, replacing episodic annual audits with an always-current savings pipeline.</t>
+        </is>
+      </c>
+      <c r="H164" s="4" t="inlineStr">
+        <is>
+          <t>Savings pipeline equal to 9-12% of addressable energy and waste spend surfaced within 10 weeks; 40 or more quantified, ROI-ranked projects identified in the diagnostic window; Leadership gained a living, data-driven savings pipeline in place of an annual audit - refreshed continuously and owned by name</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="4" t="inlineStr">
+        <is>
+          <t>MSS084</t>
+        </is>
+      </c>
+      <c r="B165" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C165" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Asset Reliability, predictive, maintenance, critical, assets, asset, sensing, remaining, useful, life, forecasting</t>
+        </is>
+      </c>
+      <c r="D165" s="4" t="inlineStr">
+        <is>
+          <t>PREDICTIVE MAINTENANCE FOR CRITICAL ASSETS</t>
+        </is>
+      </c>
+      <c r="E165" s="4" t="inlineStr">
+        <is>
+          <t>Critical assets across this manufacturer's lines - compressors, pumps, fans, motors, conveyors, and refrigeration units - were either maintained reactively after failure or serviced on fixed calendar intervals regardless of actual condition. Unplanned breakdowns caused line stoppages, emergency spare procurement, overtime, and lost output that the production schedule absorbed with difficulty. At the same time, calendar-based maintenance was over-servicing healthy assets, consuming labor and parts on equipment that did not need intervention. There was no early warning on bearing wear, imbalance, or thermal drift, and the gap between what maintenance cost and what it actually protected was invisible.</t>
+        </is>
+      </c>
+      <c r="F165" s="4" t="inlineStr">
+        <is>
+          <t>A predictive maintenance layer was deployed combining existing SCADA telemetry with targeted vibration, acoustic, and thermal sensing on the critical asset cohort. ML models analyzed the combined signal stream to detect early failure signatures, classify failure modes, and recommend specific maintenance windows - advisory to planners throughout, with no autonomous action taken. When risk thresholds were crossed, work orders were automatically created in the existing CMMS, giving planners an intervention queue ranked by risk and line impact. Maintenance shifted from firefighting and calendar-following to condition-based planning with quantified confidence in when to act.</t>
+        </is>
+      </c>
+      <c r="G165" s="4" t="inlineStr">
+        <is>
+          <t>Critical Asset Sensing: Existing SCADA telemetry augmented with vibration, acoustic, and thermal sensors on covered assets for full failure-signal capture.
+Remaining Useful Life Forecasting: ML models predict time-to-failure per asset, giving planners a quantified intervention window before failure occurs.
+Failure Mode Classification: Identifies the specific type of failure developing and recommends the appropriate maintenance action for that mode.
+CMMS Work Order Automation: Automatically creates prioritized work orders in the existing maintenance system when risk thresholds are crossed.
+Planner Risk Dashboard: Risk-ranked view of all covered assets enabling maintenance planners to sequence interventions by consequence and urgency.
+PM Interval Optimization: Replaces fixed-calendar schedules with condition-based intervals calibrated to actual asset health and operating history.</t>
+        </is>
+      </c>
+      <c r="H165" s="4" t="inlineStr">
+        <is>
+          <t>35-45% reduction in unplanned stoppages on covered assets; 20-25% reduction in maintenance cost through condition-based scheduling replacing over-maintenance of healthy equipment; ROI greater than 8:1 achieved within 12 months of deployment</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="4" t="inlineStr">
+        <is>
+          <t>MSS085</t>
+        </is>
+      </c>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C166" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Line Productivity, oee, throughput, uplift, packaging, lines, direct, line, signal, capture, automatic</t>
+        </is>
+      </c>
+      <c r="D166" s="4" t="inlineStr">
+        <is>
+          <t>OEE AND THROUGHPUT UPLIFT ON PACKAGING LINES</t>
+        </is>
+      </c>
+      <c r="E166" s="4" t="inlineStr">
+        <is>
+          <t>Lines at this manufacturer ran below nameplate capacity, but nobody could pinpoint why with confidence. Losses were buried in thousands of micro-stops, speed losses, and long changeovers that were recorded inconsistently on paper or not captured at all - meaning the most expensive minutes of downtime were also the least visible. Bottlenecks shifted by SKU and by shift, so improvement efforts targeted the problem from last week, not the one happening now, and gains from one intervention eroded before the next one began. Without a real-time loss classification layer, line teams were always reacting to what they could feel rather than what the data showed.</t>
+        </is>
+      </c>
+      <c r="F166" s="4" t="inlineStr">
+        <is>
+          <t>An OEE intelligence layer was deployed reading line controls directly through existing PLC and SCADA signals, capturing every stop and speed loss at high resolution and classifying it automatically without manual input. Dynamic bottleneck identification updated in real time as production conditions shifted, and changeover analytics surfaced specific time-reduction opportunities by SKU and shift. Root-cause Pareto charts were pushed to operator screens within the shift, so teams acted on the current loss pattern rather than waiting for end-of-day reports. No MES was replaced and no existing control system was touched.</t>
+        </is>
+      </c>
+      <c r="G166" s="4" t="inlineStr">
+        <is>
+          <t>Direct Line Signal Capture: Reads PLC and SCADA signals from existing line controls for high-resolution, second-by-second stop and speed loss logging.
+Automatic Loss Classification: Every micro-stop and speed loss classified without manual input, replacing paper-based and inconsistent recording.
+Dynamic Bottleneck Identification: Identifies the shifting constraint across the line by SKU and shift in real time as production conditions change.
+Changeover Analytics: Measures and benchmarks changeover time by SKU and shift, surfacing specific and actionable time-reduction opportunities.
+Real-Time Operator Pareto: Loss ranking by frequency and impact pushed to operator screens within the shift for targeted in-shift action.
+SKU and Shift OEE Benchmarking: Compares OEE across SKUs, shifts, and lines to identify structural performance gaps that aggregate reporting obscures.</t>
+        </is>
+      </c>
+      <c r="H166" s="4" t="inlineStr">
+        <is>
+          <t>OEE improved 6-9 points on piloted lines; Changeover time reduced 15-20%; Additional demand absorbed through throughput uplift with zero capital investment and under 8 weeks to first measurable value</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="4" t="inlineStr">
+        <is>
+          <t>MSS086</t>
+        </is>
+      </c>
+      <c r="B167" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C167" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Utilities Optimization, compressed, air, system, optimization, network, flow, pressure, analytics, leak, load</t>
+        </is>
+      </c>
+      <c r="D167" s="4" t="inlineStr">
+        <is>
+          <t>COMPRESSED AIR SYSTEM OPTIMIZATION</t>
+        </is>
+      </c>
+      <c r="E167" s="4" t="inlineStr">
+        <is>
+          <t>Compressed air at this plant - often the most expensive utility per unit of useful energy - was being generated oversized and leaking heavily, but nobody knew by how much. There was no metering on system pressure or flow, no view of total leak load, and no analysis of how compressors were being sequenced across the day. Leaks, artificial demand from overinflated pressure setpoints, and inefficient part-load compressor running were collectively wasting a significant share of what was being generated. The engineering team had a sense the system was inefficient but had no ranked list of what to fix first or what each repair was worth.</t>
+        </is>
+      </c>
+      <c r="F167" s="4" t="inlineStr">
+        <is>
+          <t>Flow and pressure analytics were deployed across the compressed air network, establishing a real baseline of consumption, leak load, and demand profile for the first time. ML-based leak load estimation quantified the total loss without requiring a physical leak detection survey, and true demand modeling identified how much pressure the system actually needed versus how much it was being forced to maintain. Compressor sequencing was optimized to eliminate inefficient part-load running, and a financially ranked repair worklist gave engineering a clear sequence to work through. The deployment model was designed from the start for replication across other sites.</t>
+        </is>
+      </c>
+      <c r="G167" s="4" t="inlineStr">
+        <is>
+          <t>Network Flow and Pressure Analytics: Continuous monitoring across the compressed air distribution network establishing a real consumption and loss baseline.
+Leak Load Estimation: ML-based quantification of total leak volume and financial cost without requiring physical leak detection surveys.
+Demand Profile Modeling: Models true compressed air demand by time of day, line, and production schedule against actual generation.
+Compressor Load Sequencing: Optimizes which compressors run and at what load, eliminating inefficient part-load operation across the generation estate.
+Pressure Setpoint Right-Sizing: Reduces system pressure to the minimum required for end-use, eliminating artificial demand across distribution points.
+Financial Impact Repair Ranking: Leak and inefficiency repair backlog ranked by cost impact, giving engineering a prioritized and financially justified action sequence.</t>
+        </is>
+      </c>
+      <c r="H167" s="4" t="inlineStr">
+        <is>
+          <t>15-22% reduction in compressed air energy on addressed scope; Full leak backlog mapped and ranked by financial impact for the first time; Compressor sequencing optimized, eliminating inefficient part-load running and reducing peak generation cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="4" t="inlineStr">
+        <is>
+          <t>MSS087</t>
+        </is>
+      </c>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C168" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Utilities Optimization, industrial, refrigeration, cooling, optimization, demand-aware, sequencing, floating, setpoint, tower, load</t>
+        </is>
+      </c>
+      <c r="D168" s="4" t="inlineStr">
+        <is>
+          <t>INDUSTRIAL REFRIGERATION AND COOLING OPTIMIZATION</t>
+        </is>
+      </c>
+      <c r="E168" s="4" t="inlineStr">
+        <is>
+          <t>Refrigeration and chilled water systems at this company ran on fixed setpoints regardless of production schedule, ambient conditions, or actual thermal load - meaning the system was always sized for worst case, even when throughput was a fraction of peak. Chillers cycled inefficiently, condensers fouled over time without triggering any alert, and there was no mechanism connecting cooling operation to what production actually needed at any given moment. A major share of plant energy was consumed at a fixed cost that bore no relationship to output, and nobody had visibility into how much of that was preventable.</t>
+        </is>
+      </c>
+      <c r="F168" s="4" t="inlineStr">
+        <is>
+          <t>An AI load-balancing and setpoint optimization layer was deployed across the cooling estate - chillers, compressors, and cooling towers - tying operation to real production demand rather than fixed worst-case parameters. Floating head-pressure and setpoint recommendations replaced static operating points, and demand-aware sequencing pre-positioned cooling capacity based on the production schedule before load arrived. Anomaly detection on chiller and condenser performance caught fouling and drift early, before efficiency losses compounded into trip risk. The system operated advisory-first above existing controls throughout.</t>
+        </is>
+      </c>
+      <c r="G168" s="4" t="inlineStr">
+        <is>
+          <t>Demand-Aware Cooling Sequencing: Ties chiller and compressor operation to the actual production schedule, eliminating worst-case fixed setpoint running.
+Floating Setpoint Optimization: Continuously recommends optimal head pressure and temperature setpoints based on live load and ambient conditions.
+Cooling Tower Load Balancing: Distributes load across cooling towers to maximize efficiency and minimize energy per unit of cooling delivered.
+Condenser Fouling Detection: Anomaly detection on chiller and condenser performance identifying fouling before it compounds into efficiency loss or trip risk.
+Cooling Performance Benchmarking: Continuous measurement of cooling system efficiency against baseline across all chillers, compressors, and towers.
+Production Schedule Integration: Reads the production plan to pre-position cooling capacity, eliminating reactive ramp-up and associated energy spikes.</t>
+        </is>
+      </c>
+      <c r="H168" s="4" t="inlineStr">
+        <is>
+          <t>12-18% reduction in refrigeration energy on the addressed cooling estate; Earlier detection of condenser fouling and performance drift, reducing unplanned cooling trips; Cooling operation brought into real-time alignment with production demand, ending fixed-setpoint overconsumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="4" t="inlineStr">
+        <is>
+          <t>MSS088</t>
+        </is>
+      </c>
+      <c r="B169" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C169" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Quality and Yield Optimization, fill, weight, giveaway, reduction, per-head, distribution, modeling, drift, detection, compliant</t>
+        </is>
+      </c>
+      <c r="D169" s="4" t="inlineStr">
+        <is>
+          <t>FILL WEIGHT AND GIVEAWAY REDUCTION</t>
+        </is>
+      </c>
+      <c r="E169" s="4" t="inlineStr">
+        <is>
+          <t>Every pack leaving this manufacturer's filling lines carried a small amount of extra product - an intentional safety margin above the declared net weight, held wide to avoid underweight compliance breaches. Across millions of packs per shift, the cumulative giveaway was a substantial recurring cost that appeared nowhere on any report because it was treated as normal. Fill distributions were wide because individual filling heads varied and drifted across shifts, and the team had no per-head view of where the variance was coming from. Tightening the margin manually felt like regulatory risk, so nobody touched it - and the giveaway continued, invisibly, on every line.</t>
+        </is>
+      </c>
+      <c r="F169" s="4" t="inlineStr">
+        <is>
+          <t>Fill analytics were deployed combining checkweigher and fill-head data into individual per-head distribution models, giving the team its first precise view of how each head actually performed and how it drifted across shifts. ML drift detection monitored every head continuously, flagging deviation before it widened the distribution or pushed toward the underweight limit. Statistically safe tighter setpoints were recommended for operator confirmation - never applied autonomously - with a compliance guardrail that made the underweight limit inviolable in every recommendation. The method was standardized for deployment across all filling lines after single-line validation.</t>
+        </is>
+      </c>
+      <c r="G169" s="4" t="inlineStr">
+        <is>
+          <t>Per-Head Fill Distribution Modeling: Combines checkweigher and fill-head data to characterize each head's individual performance, variance, and drift pattern.
+ML Drift Detection: Monitors every filling head across shifts and flags drift patterns before they widen the distribution or approach compliance limits.
+Compliant Setpoint Recommendations: Calculates statistically safe tighter targets that reduce giveaway while keeping every recommendation above the underweight limit.
+Underweight Compliance Guardrails: Enforces a regulatory floor on all setpoint recommendations, making compliance breach impossible by design.
+Operator-Confirmed Closed Loop: All setpoint changes require operator confirmation before adjustment, keeping quality decisions human-gated throughout.
+Cross-Line Replication Framework: Methodology standardized for deployment across all filling lines after single-line pilot validation.</t>
+        </is>
+      </c>
+      <c r="H169" s="4" t="inlineStr">
+        <is>
+          <t>0.8-1.4% reduction in average giveaway per pack; 100% net-weight compliance maintained throughout without exception; Six-figure annual saving per line with the methodology replicable across all filling lines in the network</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>MSS089</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C170" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Financial and Operational Control, operational, loss, margin, leakage, intelligence, real-time, category, tracking, predictive, shortage</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>OPERATIONAL LOSS AND MARGIN LEAKAGE INTELLIGENCE</t>
+        </is>
+      </c>
+      <c r="E170" s="4" t="inlineStr">
+        <is>
+          <t>Margin was leaking across this manufacturer in dozens of small, disconnected ways - scrap and rework, excess and obsolete inventory, unplanned downtime, expedited freight, off-catalog spend, and price and contract variance - each owned by a different team and invisible until month-end. No single system tied these categories together, and by the time the variance appeared in the P&amp;L, the underlying decisions were weeks old and impossible to reverse. Every month-end brought surprises that were, in retrospect, entirely predictable from operational data that existed but was never connected. Leadership was consistently managing to outcomes they could not have seen coming, because nobody had built the view that would have shown them early enough to act.</t>
+        </is>
+      </c>
+      <c r="F170" s="4" t="inlineStr">
+        <is>
+          <t>An operational intelligence layer was deployed above the existing ERP, tracking configurable loss categories in near-real-time and converting operational signals into owned, time-bound actions with named accountability. Predictive shortage and disruption signals were drawn from operational and supplier data, contract-price compliance was checked on every purchase order line at the moment of commitment, and scenario simulation allowed finance and operations to model EBITDA impact before choosing a recovery path. The platform augmented the ERP entirely - no replacement, no migration, no disruption to existing workflows.</t>
+        </is>
+      </c>
+      <c r="G170" s="4" t="inlineStr">
+        <is>
+          <t>Real-Time Loss Category Tracking: Configurable waste categories tracked in near-real-time across scrap, rework, inventory, downtime, freight, and spend simultaneously.
+Predictive Shortage and Disruption Signals: Forward-looking signals from operational and supplier data flagging emerging risk before it materializes as loss.
+Owned Escalation Workflows: Auto-created escalation tasks with named owners and SLAs ensuring every flagged loss has a responsible action and a deadline.
+Contract Price Compliance Checking: Every purchase order line checked against contracted rates at the moment of commitment, flagging variance before payment.
+EBITDA Scenario Simulation: Models the financial impact of alternative recovery paths before a decision is made, replacing instinct with evidence.
+Loss Pareto and Structured Problem Solving: Built-in ranking of loss drivers with a structured 8D framework for root cause identification and resolution.</t>
+        </is>
+      </c>
+      <c r="H170" s="4" t="inlineStr">
+        <is>
+          <t>2-4% of addressable operational loss recovered in the first 2 quarters; 15-20% reduction in scrap and rework on addressed scope; Month-end loss surprises largely eliminated through in-month visibility, named ownership, and time-bound accountability</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="4" t="inlineStr">
+        <is>
+          <t>MSS090</t>
+        </is>
+      </c>
+      <c r="B171" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C171" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Utilities Optimization, boiler, steam, thermal, utilities, optimization, efficiency, monitoring, combustion, drift, detection</t>
+        </is>
+      </c>
+      <c r="D171" s="4" t="inlineStr">
+        <is>
+          <t>BOILER AND STEAM THERMAL UTILITIES OPTIMIZATION</t>
+        </is>
+      </c>
+      <c r="E171" s="4" t="inlineStr">
+        <is>
+          <t>This manufacturer's boiler and steam systems were run largely on operator experience, with no analytics connecting fuel consumption to actual thermal demand. Combustion efficiency drifted over time without triggering any alert, condensate recovery was poor and going unmeasured, and recoverable heat was being vented to atmosphere as a matter of course. The losses were real but invisible: without a baseline and without monitoring, the plant had no way to quantify how much efficiency had quietly eroded or where to start recovering it. Fuel cost was treated as a fixed operating reality rather than a variable with recoverable opportunity inside it.</t>
+        </is>
+      </c>
+      <c r="F171" s="4" t="inlineStr">
+        <is>
+          <t>Combustion and steam system analytics were deployed monitoring boiler efficiency continuously, correlating steam demand against fuel consumption to surface unexplained gaps, and flagging combustion drift before it compounded into significant cost. Excess air monitoring enabled real-time combustion optimization recommendations, and condensate and waste-heat recovery opportunities were identified and quantified for the engineering team to action. The system operated entirely in an advisory capacity, producing structured recommendations rather than autonomous adjustments, and was sized to provide payback inside the diagnostic engagement window.</t>
+        </is>
+      </c>
+      <c r="G171" s="4" t="inlineStr">
+        <is>
+          <t>Boiler Efficiency Monitoring: Continuous tracking of combustion efficiency and excess air across all boilers with specific optimization recommendations.
+Combustion Drift Detection: Alerts when combustion performance drifts below target, enabling corrective action before efficiency loss compounds.
+Condensate Recovery Opportunity Detection: Identifies where condensate is being lost rather than returned, quantifying the fuel and water cost of each loss point.
+Waste Heat Recovery Identification: Surfaces recoverable heat currently vented to atmosphere and quantifies the fuel saving achievable from recovery.
+Steam Demand and Fuel Correlation: Connects fuel consumption to actual thermal demand, flagging unexplained gaps as recoverable loss signals.
+Engineering Advisory Reporting: All findings delivered as structured, actionable engineering recommendations with quantified financial impact.</t>
+        </is>
+      </c>
+      <c r="H171" s="4" t="inlineStr">
+        <is>
+          <t>6-11% reduction in thermal fuel cost on addressed boiler and steam scope; Combustion efficiency recovered from drift to target levels through continuous monitoring and corrective action; Condensate and heat recovery improved, cutting make-up water and fuel costs simultaneously</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="4" t="inlineStr">
+        <is>
+          <t>MSS091</t>
+        </is>
+      </c>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C172" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Utilities and Sustainability, water, effluent, optimization, plant-wide, balance, analytics, leak, loss, detection, cip</t>
+        </is>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t>WATER AND EFFLUENT OPTIMIZATION</t>
+        </is>
+      </c>
+      <c r="E172" s="4" t="inlineStr">
+        <is>
+          <t>Water at this plant was drawn, used, and discharged with limited sub-metering, making it almost impossible to locate losses, leaks, or inefficient CIP and wash cycles from available data. Effluent treatment was energy-intensive and ran at a fixed dosing rate regardless of actual load, consuming chemical and power inputs that bore no relationship to what the treatment system was handling on any given day. With water scarcity raising both the unit cost and the regulatory risk of overconsumption, the plant needed a water balance - but building one manually from the instrumentation available was not feasible. The team knew they were wasting water; they had no way to prove where or by how much.</t>
+        </is>
+      </c>
+      <c r="F172" s="4" t="inlineStr">
+        <is>
+          <t>A water balance analytics layer was deployed spanning intake, process use, CIP, and effluent treatment, establishing a complete plant-wide water flow model from existing instrumentation for the first time. Leak and loss detection identified waste streams across the network and quantified each by cost, CIP cycle optimization reduced water and time per clean, and effluent treatment energy and chemical dosing were optimized against actual daily load rather than fixed parameters. Anomaly detection flagged treatment performance deviations before they created compliance risk, and water intensity was benchmarked by line and shift to track progress continuously.</t>
+        </is>
+      </c>
+      <c r="G172" s="4" t="inlineStr">
+        <is>
+          <t>Plant-Wide Water Balance Analytics: Establishes a complete water flow model across intake, process, CIP, and effluent treatment from existing instrumentation.
+Leak and Loss Detection: Identifies where water is being lost across the distribution network and quantifies each loss stream by daily cost.
+CIP Cycle Optimization: Analyzes cleaning-in-place cycles to reduce water consumption and cycle time without compromising hygiene or validation standards.
+Effluent Treatment Load Optimization: Optimizes energy and chemical dosing against actual daily effluent load, replacing fixed-rate dosing with demand-based operation.
+Treatment Anomaly Detection: Flags abnormal effluent treatment performance before it escalates into compliance risk or chemical cost overrun.
+Water Intensity Benchmarking: Continuous measurement of water use per unit of output by line and shift, tracking improvement and surfacing new reduction opportunities.</t>
+        </is>
+      </c>
+      <c r="H172" s="4" t="inlineStr">
+        <is>
+          <t>15-22% reduction in freshwater draw on addressed process scope; Effluent treatment energy and chemical dosing cost reduced through load-based optimization; Plant-wide water balance made visible for the first time, turning scarcity risk from an accepted exposure into a managed and improving metric</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="4" t="inlineStr">
+        <is>
+          <t>MSS092</t>
+        </is>
+      </c>
+      <c r="B173" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C173" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Quality Assurance, inline, vision, quality, inspection, coverage, multi-type, defect, classification, real-time, reject</t>
+        </is>
+      </c>
+      <c r="D173" s="4" t="inlineStr">
+        <is>
+          <t>INLINE VISION QUALITY INSPECTION</t>
+        </is>
+      </c>
+      <c r="E173" s="4" t="inlineStr">
+        <is>
+          <t>Packaging defects at this manufacturer - seal integrity failures, label and print errors, fill level issues, cap and closure faults, code and date legibility problems, and foreign objects on the belt - were caught only through sampling, which meant a statistically predictable number of defective packs reached customers every period. Manual inspection could not keep pace at line speed, and sampling by definition left the vast majority of packs uninspected. Rework volumes were rising, customer complaint patterns were repeating, and the quality team was always investigating last week's escape rather than preventing today's.</t>
+        </is>
+      </c>
+      <c r="F173" s="4" t="inlineStr">
+        <is>
+          <t>Inline computer vision was deployed on packaging lines providing 100% inspection coverage at full line speed across multiple defect types simultaneously, without touching any existing control system. Quality-critical and safety-critical dispositions were kept under human approval with a complete audit trail, so the system augmented QA judgment rather than replacing it on consequential decisions. Defect trend analytics aggregated detection data over time and traced recurring patterns back to upstream process conditions, turning individual defect catches into inputs to permanent process fixes.</t>
+        </is>
+      </c>
+      <c r="G173" s="4" t="inlineStr">
+        <is>
+          <t>100% Inline Inspection Coverage: Computer vision inspects every pack at line speed across multiple defect types simultaneously, with no sampling gap.
+Multi-Type Defect Classification: ML classifies seal, label, print, fill level, closure, code, and foreign object defects in real time without manual review.
+Real-Time Reject and Operator Alert: Immediate rejection signal and line alert on detected defects before packs advance to downstream packing or palletizing.
+Defect Trend Analytics: Aggregates detection data over time to identify patterns and trace recurring defects back to upstream process root causes.
+Human-Gated Critical Dispositions: Quality-critical and safety-critical decisions remain under human approval with a complete, time-stamped audit trail.
+Upstream Process Feedback Loop: Defect trend data linked back to process parameters, enabling permanent fixes rather than ongoing reject-and-replace cycles.</t>
+        </is>
+      </c>
+      <c r="H173" s="4" t="inlineStr">
+        <is>
+          <t>40-55% reduction in defect escapes on covered defect types; 20-30% reduction in rework driven by earlier in-line detection; 100% inspection coverage achieved across all inspected lines, from a sampling-only baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="4" t="inlineStr">
+        <is>
+          <t>MSS093</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C174" s="4" t="inlineStr">
+        <is>
+          <t>Process Manufacturing, Capital Project Governance, capital, project, cost, schedule, intelligence, multi-source, data, consolidation, slippage, prediction</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>CAPITAL PROJECT COST AND SCHEDULE INTELLIGENCE</t>
+        </is>
+      </c>
+      <c r="E174" s="4" t="inlineStr">
+        <is>
+          <t>Large capital projects at this manufacturer consistently overran on cost and schedule, but the problems only surfaced late - after commitments had been made, vendors had been paid, and construction had locked in the outcome. Project data was scattered across schedules, purchase orders, vendor update emails, and progress reports, and nobody had a consolidated view that could predict slippage early enough to act on it. Leadership was approving next-phase funding without reliable visibility into whether the current phase was on track, and the first sign of a problem was usually a contractor requesting a variation or a delivery sliding past a milestone.</t>
+        </is>
+      </c>
+      <c r="F174" s="4" t="inlineStr">
+        <is>
+          <t>A project intelligence layer was deployed consolidating schedule, cost, procurement, and vendor progress data across the entire capital portfolio into a single early-warning view. ML risk prediction for cost and schedule slippage ran continuously across all active projects, flagging risk weeks before it became a confirmed overrun. Vendor and purchase order variance was tracked against contracted terms as commitments were made, milestone risk dashboards gave project leadership a daily view of exposure across all concurrent projects, and automated escalation ensured risks reached decision-makers early enough to matter.</t>
+        </is>
+      </c>
+      <c r="G174" s="4" t="inlineStr">
+        <is>
+          <t>Multi-Source Project Data Consolidation: Connects schedule, cost, procurement, vendor updates, and progress reports into a single consolidated project view.
+ML Cost and Schedule Slippage Prediction: Predicts overrun risk weeks in advance, giving project leadership time to intervene before commitments are locked.
+Vendor and PO Variance Tracking: Monitors vendor performance and purchase order commitments against contracted terms continuously as work progresses.
+Milestone Risk Dashboards: Visual tracking of milestone status with risk scoring and automated escalation to named project decision-makers.
+Early Warning Escalation: Automated alerts routed to responsible leads when risk thresholds are crossed on cost, schedule, or vendor delivery.
+Portfolio-Level Capital Visibility: Single consolidated view across all concurrent capital projects enabling cross-project prioritization and resource decisions.</t>
+        </is>
+      </c>
+      <c r="H174" s="4" t="inlineStr">
+        <is>
+          <t>10-18% reduction in cost and schedule overrun on covered capital projects; Risk visibility shifted from post-overrun discovery to early-enough-to-act alerts; Capital approval decisions made with reliable, portfolio-wide visibility for the first time</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="4" t="inlineStr">
+        <is>
+          <t>MSS094</t>
+        </is>
+      </c>
+      <c r="B175" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C175" s="4" t="inlineStr">
+        <is>
+          <t>Manufacturing, Aftersales and Field Service Operations, unified, field, service, orchestration, multi-partner, data, normalization, partner, capability, mapping</t>
+        </is>
+      </c>
+      <c r="D175" s="4" t="inlineStr">
+        <is>
+          <t>UNIFIED FIELD SERVICE ORCHESTRATION</t>
+        </is>
+      </c>
+      <c r="E175" s="4" t="inlineStr">
+        <is>
+          <t>Post-sales service at this manufacturer ran across multiple third-party partners - each operating from their own CRM, portal, or email-based update system - with no unified view connecting them. Service status, technician availability, and job completion data required manual reconciliation daily by a central team spending hours chasing updates that should have been automatic. Demand spikes went undetected until SLA breaches had already occurred, because no signal connected incoming service volume to available field capacity across the partner network in real time. Customer communication depended entirely on individual partner responsiveness, meaning customers received updates inconsistently, in whatever language the local partner happened to use, if they received them at all.</t>
+        </is>
+      </c>
+      <c r="F175" s="4" t="inlineStr">
+        <is>
+          <t>A unified field service orchestration layer was deployed to ingest and normalize updates from every partner CRM, portal, and email channel into a single operational view without requiring any partner to change their systems. Capability mapping across the partner network made technician skills, coverage zones, and real-time capacity visible for job routing decisions that previously relied on phone calls. A demand forecasting engine processed incoming service signals to flag emerging volume before it hit SLA thresholds, giving operations time to rebalance capacity across partners. A proactive customer communication layer on WhatsApp triggered structured status updates automatically at every job milestone in the customer's preferred Indian language, removing partner action as a dependency in the customer experience.</t>
+        </is>
+      </c>
+      <c r="G175" s="4" t="inlineStr">
+        <is>
+          <t>Multi-Partner Data Normalization: Ingests and standardizes updates from every partner CRM, portal, and email feed into one live operational view without partner system changes.
+Partner Capability Mapping: Maps technician skills, coverage zones, and real-time capacity across the full network, enabling intelligent job routing.
+Demand Forecasting: Detects emerging service volume patterns across regions and product lines before they breach SLA thresholds.
+Proactive Customer Communication: Automatically triggers WhatsApp status updates at every job milestone without relying on partner action.
+Multilingual Communication Engine: Supports all major Indian languages natively, eliminating language and consistency gaps in customer-facing updates.
+Unified Service Operations Dashboard: Consolidates job status, partner performance, SLA risk, and regional demand into a single real-time leadership view.</t>
+        </is>
+      </c>
+      <c r="H175" s="4" t="inlineStr">
+        <is>
+          <t>60-70% reduction in manual reconciliation effort across partner service networks; Customer update delays cut from hours to minutes through system-triggered communication; Service leadership shifted from reactive SLA firefighting to proactive, demand-signal-driven capacity planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="4" t="inlineStr">
+        <is>
+          <t>MSS095</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>MS Solution</t>
+        </is>
+      </c>
+      <c r="C176" s="4" t="inlineStr">
+        <is>
+          <t>Life Sciences, Quality Assurance and Compliance, coa, parameter, efficiency, tracker, failure, analytics, near-miss, detection, product, risk</t>
+        </is>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t>COA PARAMETER EFFICIENCY TRACKER</t>
+        </is>
+      </c>
+      <c r="E176" s="4" t="inlineStr">
+        <is>
+          <t>Quality teams at this pharmaceutical manufacturer investigated out-of-specification failures one batch at a time, with no systematic way to identify whether the same parameter was drifting across multiple products or whether a pattern of near-misses was accumulating toward a future failure. The investigation process was intensive, manual, and reactive - consuming significant analyst hours on each event while leaving the next one just as unpredictable as the last. Parameters drifting toward specification limits went undetected because the data lived in COA records, LIMS, and ERP systems that were never analyzed together. Batch release delays, rework cycles, and customer escalations were absorbed as the cost of doing business in a complex quality environment, when the signals to prevent them had been there all along.</t>
+        </is>
+      </c>
+      <c r="F176" s="4" t="inlineStr">
+        <is>
+          <t>An AI-powered analytics platform was deployed continuously analyzing COA, LIMS, ERP, and supplier data together to surface quality risk before it materialized as a failure. Parameter behavior was tracked across the entire product portfolio, with near-miss detection flagging parameters drifting toward specification limits before they triggered an out-of-specification event. Dynamic product risk scores were generated from process capability, trend stability, and historical failure data, and failure correlations with suppliers, equipment, shifts, and process conditions were surfaced automatically for quality team review. Automated SPC monitoring and one-click audit reporting replaced the manual assembly of trend data that had previously consumed analyst time before every customer audit or regulatory review.</t>
+        </is>
+      </c>
+      <c r="G176" s="4" t="inlineStr">
+        <is>
+          <t>Parameter Failure Analytics: Tracks out-of-specification frequency across products and parameters, identifying recurring failure patterns and high-risk areas continuously.
+Near-Miss Detection: Flags parameters drifting toward specification limits before an out-of-specification event occurs, enabling intervention before failure.
+Product Risk Scoring: Generates dynamic risk scores from process capability, trend stability, and historical failure data across the full product portfolio.
+Root Cause Correlation Engine: Correlates failures with suppliers, equipment, shifts, and process conditions, surfacing probable root-cause hypotheses automatically.
+Automated SPC and Process Monitoring: Real-time SPC charts and continuous Cpk and Ppk monitoring for every critical quality parameter across all products.
+Audit and Compliance Reporting: One-click generation of comprehensive trend reports for customer audits, regulatory reviews, and internal quality assessments.</t>
+        </is>
+      </c>
+      <c r="H176" s="4" t="inlineStr">
+        <is>
+          <t>Rs 1.0-2.5 crore reduction in out-of-specification investigation cost; Batch release cycles accelerated by 1-2 days through proactive risk detection replacing reactive investigation; Quality management shifted from batch-by-batch reactive investigation to continuous, portfolio-wide predictive intelligence</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I161"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>

</xml_diff>